<commit_message>
docs: update Phase 2 estimate and internal roadmap
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SCION_Phase2_Estimate.xlsx
+++ b/docs/SCION_Phase2_Estimate.xlsx
@@ -648,30 +648,30 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -989,7 +989,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="40"/>
@@ -998,7 +998,7 @@
       <c r="E1" s="40"/>
     </row>
     <row r="2" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="41" t="s">
         <v>98</v>
       </c>
       <c r="B2" s="40"/>
@@ -1025,7 +1025,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="44" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="40"/>
@@ -1085,7 +1085,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="43" t="s">
+      <c r="A9" s="44" t="s">
         <v>18</v>
       </c>
       <c r="B9" s="40"/>
@@ -1145,7 +1145,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="43" t="s">
+      <c r="A13" s="44" t="s">
         <v>31</v>
       </c>
       <c r="B13" s="40"/>
@@ -1262,7 +1262,7 @@
     </row>
     <row r="21" spans="1:5" ht="6" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
     <row r="22" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="47" t="s">
+      <c r="A22" s="42" t="s">
         <v>54</v>
       </c>
       <c r="B22" s="40"/>
@@ -1273,7 +1273,7 @@
       <c r="E22" s="23"/>
     </row>
     <row r="23" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="47" t="s">
+      <c r="A23" s="42" t="s">
         <v>56</v>
       </c>
       <c r="B23" s="40"/>
@@ -1284,7 +1284,7 @@
       <c r="E23" s="23"/>
     </row>
     <row r="24" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="44" t="s">
+      <c r="A24" s="45" t="s">
         <v>58</v>
       </c>
       <c r="B24" s="40"/>
@@ -1297,7 +1297,7 @@
       </c>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="45" t="s">
+      <c r="A26" s="39" t="s">
         <v>60</v>
       </c>
       <c r="B26" s="40"/>
@@ -1306,7 +1306,7 @@
       <c r="E26" s="40"/>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" s="45" t="s">
+      <c r="A27" s="39" t="s">
         <v>61</v>
       </c>
       <c r="B27" s="40"/>
@@ -1315,7 +1315,7 @@
       <c r="E27" s="40"/>
     </row>
     <row r="28" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" s="45" t="s">
+      <c r="A28" s="39" t="s">
         <v>62</v>
       </c>
       <c r="B28" s="40"/>
@@ -1324,7 +1324,7 @@
       <c r="E28" s="40"/>
     </row>
     <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="45" t="s">
+      <c r="A29" s="39" t="s">
         <v>63</v>
       </c>
       <c r="B29" s="40"/>
@@ -1334,6 +1334,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A9:E9"/>
     <mergeCell ref="A29:E29"/>
     <mergeCell ref="A26:E26"/>
     <mergeCell ref="A2:E2"/>
@@ -1341,11 +1346,6 @@
     <mergeCell ref="A28:E28"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A27:E27"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1366,7 +1366,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="43" t="s">
         <v>64</v>
       </c>
       <c r="B1" s="40"/>
@@ -1379,7 +1379,7 @@
       <c r="A3" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="46" t="s">
         <v>66</v>
       </c>
       <c r="C3" s="40"/>
@@ -1391,7 +1391,7 @@
       <c r="A4" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="B4" s="39" t="s">
+      <c r="B4" s="46" t="s">
         <v>68</v>
       </c>
       <c r="C4" s="40"/>
@@ -1403,7 +1403,7 @@
       <c r="A5" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="46" t="s">
         <v>99</v>
       </c>
       <c r="C5" s="40"/>
@@ -1415,7 +1415,7 @@
       <c r="A6" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="B6" s="39" t="s">
+      <c r="B6" s="46" t="s">
         <v>100</v>
       </c>
       <c r="C6" s="40"/>
@@ -1427,7 +1427,7 @@
       <c r="A7" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="39" t="s">
+      <c r="B7" s="46" t="s">
         <v>72</v>
       </c>
       <c r="C7" s="40"/>
@@ -1439,7 +1439,7 @@
       <c r="A8" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="39" t="s">
+      <c r="B8" s="46" t="s">
         <v>74</v>
       </c>
       <c r="C8" s="40"/>
@@ -1451,7 +1451,7 @@
       <c r="A9" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="B9" s="39" t="s">
+      <c r="B9" s="46" t="s">
         <v>76</v>
       </c>
       <c r="C9" s="40"/>
@@ -1544,7 +1544,7 @@
     </row>
     <row r="17" spans="1:4" ht="10" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
     <row r="18" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="41" t="s">
+      <c r="A18" s="47" t="s">
         <v>97</v>
       </c>
       <c r="B18" s="40"/>

</xml_diff>